<commit_message>
test bulk categorization and customer/sales imports
</commit_message>
<xml_diff>
--- a/Frontend/assets/careloop_customer_import_template.xlsx
+++ b/Frontend/assets/careloop_customer_import_template.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -574,22 +574,43 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Customer Type - Optional. Must be 'new' or 'active'. Defaults to 'new' if left blank.</t>
+          <t>Customer Type - Optional. Must be 'new', 'active', or 'inactive'. Defaults to 'new' if left blank.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Has Purchased - Optional. Enter 'yes' or 'no'. Defaults to 'no' if left blank.</t>
+          <t xml:space="preserve">  - New: a customer you have not followed up with much yet.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Active: an existing customer, follows a shorter 7-day follow-up cycle.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Inactive: stops follow-up reminders entirely for this customer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Has Purchased - Optional. Enter 'yes' or 'no'. Defaults to 'no' if left blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Delete the example row (row 2 on the Customers sheet) before uploading your own data.</t>
         </is>

</xml_diff>